<commit_message>
#381 Added pre allocation tab to template and upload
</commit_message>
<xml_diff>
--- a/wwwroot/templates/PrismAdjustmentsTemplate.xlsx
+++ b/wwwroot/templates/PrismAdjustmentsTemplate.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\DaleSandboxApp2\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7FE5732-E007-42F5-9983-B72F2266FDFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A82BD54F-688D-4045-AD69-2AA5AC404363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-18885" yWindow="1995" windowWidth="21600" windowHeight="11295" activeTab="3" xr2:uid="{8129F872-A949-4512-A997-996043680CD8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{8129F872-A949-4512-A997-996043680CD8}"/>
   </bookViews>
   <sheets>
     <sheet name="ORI Policies" sheetId="1" r:id="rId1"/>
     <sheet name="Incurred Claims" sheetId="2" r:id="rId2"/>
     <sheet name="Ultimate Claims" sheetId="3" r:id="rId3"/>
     <sheet name="Allocated Recoveries and RIPs" sheetId="4" r:id="rId4"/>
+    <sheet name="Claims By Event" sheetId="5" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Allocated Recoveries and RIPs'!$A$1:$O$1</definedName>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="84">
   <si>
     <t>ORIPillar</t>
   </si>
@@ -285,6 +286,18 @@
   </si>
   <si>
     <t>UltimateBasisRIPs</t>
+  </si>
+  <si>
+    <t>ContractCcy</t>
+  </si>
+  <si>
+    <t>IsCommuted</t>
+  </si>
+  <si>
+    <t>ActualRecoveriesInSettCcy</t>
+  </si>
+  <si>
+    <t>ActualRIPsInSettCcy</t>
   </si>
 </sst>
 </file>
@@ -339,13 +352,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="47" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1086,4 +1100,94 @@
   <autoFilter ref="A1:O1" xr:uid="{386E106E-05F4-434C-B5A3-F84DB75A17FA}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEC3ACEF-DB3B-43D7-A3E4-A79E65E26FD8}">
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="24" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D2" s="6"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D3" s="6"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D4" s="6"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D5" s="6"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D6" s="6"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D7" s="6"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D8" s="6"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="D9" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Processing month for adjustments
</commit_message>
<xml_diff>
--- a/wwwroot/templates/PrismAdjustmentsTemplate.xlsx
+++ b/wwwroot/templates/PrismAdjustmentsTemplate.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\repos\DaleSandboxApp2\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A82BD54F-688D-4045-AD69-2AA5AC404363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC998741-4EC7-475E-9DCB-161C4EB16EBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{8129F872-A949-4512-A997-996043680CD8}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{8129F872-A949-4512-A997-996043680CD8}"/>
   </bookViews>
   <sheets>
     <sheet name="ORI Policies" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Allocated Recoveries and RIPs'!$A$1:$O$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Claims By Event'!$A$1:$N$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Incurred Claims'!$A$1:$AR$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ORI Policies'!$A$1:$T$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Ultimate Claims'!$A$1:$I$2</definedName>
@@ -1188,6 +1189,7 @@
       <c r="D9" s="6"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:N9" xr:uid="{AEC3ACEF-DB3B-43D7-A3E4-A79E65E26FD8}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>